<commit_message>
Underclassman watch: 3 sources, 30-min alerts, workbook sheet
underclass_watch.py watches the underclassmen-opportunities repo
(freshman/sophomore internships, programs, research), the
sndsh404/summer-2027-internships community list (tech+US filtered),
and Extern's verified underclassmen program directory (STEP, Explore,
Ignite, Propel, TEIP - with app windows). Runs inside the Simplify
workflow every 30 min; new rows alert by email+push; 158 rows
baselined and rendered as the 'Underclassman programs' sheet in
InternWatch.xlsx. Also: title veto understands negation ('Ops, Not
SWE' no longer passes as SWE).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/InternWatch.xlsx
+++ b/InternWatch.xlsx
@@ -1,18 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Watchlist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="No formal program" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="LinkedIn outreach" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="No formal program" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LinkedIn outreach" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Underclassman programs" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Watchlist'!$A$2:$K$411</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Underclassman programs'!$A$2:$F$160</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -34960,4 +34962,4825 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F160"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Freshman/sophomore programs and postings (STEP/Explore/Ignite-style). Apply to these with the Class of 2029 graduation date. Sources: underclassmen-opportunities + summer-2027-internships GitHub repos, Extern's verified directory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Program / role</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Window / location / posted</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Source section</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Propel</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Both · 12 wks</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Aug-Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Future Engineer</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Freshman · 10-12 wks</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Sophomore Analyst</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Bank of America</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Sophomore · 10 wks</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Sep-Nov 2026</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>First Year Insights</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Bloomberg</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Freshman · 1 day + virtual</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Spring 2027</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Rising Fellows</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Bridgewater</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Sophomore · 3-8 wks</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Dec 2026-Jan 2027</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>TEIP</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Both · 10 wks</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Dec 2026-Jan 2027</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Citadel</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Sophomore · 11 wks</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Oct-Nov 2026</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Discover Citadel</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Citadel</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Both · 2 days</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Fellowships</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>D.E. Shaw</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Sophomore · 3 days</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Spring 2027</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>SWE Intern</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Dropbox</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Sophomore · 12 wks</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Thrive</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Duolingo</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Sophomore · 10 wks</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Late Sep 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Pathfinder</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Both · 12 wks</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>LINK</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Five Rings</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Sophomore · 5 days</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Spring 2027</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>ASDI</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Both · 12 wks</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Late Sep-Oct 2026 (2-4 wk window)</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>WiTTI</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>HRT</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Both (women + NB) · 2-4 wks (Jan)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>FTTP</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Jane Street</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Freshman · Few days</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Jul-Aug 2026</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>JSIP</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Jane Street</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Both · Multi-week</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Fellowship</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Sophomore · 5 wks</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Nov 2026-Jan 2027</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>First Play</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Both · 12 wks</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Late Nov 2026 (2-wk window)</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Explore</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Both · 12 wks</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Sep-Oct 2026</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Fellowship</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>MLH</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>All years · 12 wks</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Early Insights</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Morgan Stanley</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Sophomore · Short</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Feb-Mar 2027</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Ignite</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Both · 12 wks</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Oct 2026 (2-wk window)</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>FutureFocus</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Optiver</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Both · 5 days</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Accelerate</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Palantir</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Soph + Junior · 10-12 wks</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Aug-Oct 2026</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>SWE Intern</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Both · 10 wks</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Futureforce Launchpad</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Sophomore · 10 wks</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Oct 2026-Feb 2027</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Tech Developer</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Both (URM) · 6 weeks</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Jan-Mar 2027</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Discovery Day</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>SIG</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Both · 2 days</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Freshman SWE</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Two Sigma</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Freshman · 10-12 wks</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Jul-Aug 2026</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>UberSTAR</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Both · 10-12 wks</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Sep-Dec 2026</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Wells Fargo</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Sophomore · 6-8 wks</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Sep-Oct 2026</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Verified directory (Extern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>AI Builder Intern (Open to All Undergrads; No Class-Year Gate) — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>San Francisco, CA Jun 17, 2026</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Internships</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (Summer 2027, Python / C++ / Full Stack / C# .NET)</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Akuna Capital</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr"/>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Chicago, IL 2026-07-14</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (apps reviewed from Aug 2026) 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Anduril</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr"/>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Costa Mesa, CA (multiple US) 2026-06-11</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Aquatic Capital</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr"/>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Chicago, IL 2026-04-02</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Quantitative Developer Intern</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Arrowstreet Capital</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr"/>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Boston, MA 2026-07-09</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern (Spring 2027)</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>ASM</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr"/>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern I (Summer 2027) 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>BAE Systems</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr"/>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Nashua, NH 2026-07-14</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Global Technology Summer Analyst, Cybersecurity Analyst 🛂</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Bank of America</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>multiple US 2026-06-28</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Global Technology Summer Analyst, Business Analyst 🛂</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Bank of America</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>multiple US 2026-06-28</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Software Developer Intern (Spring 2027) 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Blue Origin</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr"/>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Seattle, WA (multiple US) 2026-06-10</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Avionics Software Intern (Spring 2027) 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Blue Origin</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Seattle, WA (multiple US) 2026-06-10</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern (Summer 2027) 🛂</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Circleback</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>San Francisco, CA 2026-06-16</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Future Intern, Early Interest (Summer 2027, Software / AI/ML / Cyber) 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>CloudFit Software</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr"/>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Lynchburg, VA -</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern / Research Intern, Interpretability (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>CTGT</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr"/>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>San Francisco, CA 2026-06-27</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Quantitative Developer Intern</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Cubist Systematic Strategies</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr"/>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY -</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Software Developer Intern</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>D. E. Shaw</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr"/>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY 2026-04-29</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Systems Engineering Intern</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>D. E. Shaw</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr"/>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY -</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineering Intern ⏳</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>DimeHealth AI</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr"/>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY -</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Information Technology Intern (2027 Summer) 🛂</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>DTCC</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr"/>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Jersey City, NJ (multiple US) 2026-07-08</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Ellipsis Labs</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr"/>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY 2026-03-27</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Software Developer Intern ⏳</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr"/>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Verona, WI -</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Software Developer Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Five Rings</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr"/>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY 2026-07-15</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Digital Technology Intern (Spring 2027)</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>GE Appliances</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr"/>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Louisville, KY 2026-06-01</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern, BS (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr"/>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Mountain View, CA (multiple US) 2026-07-20</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern (Summer 2027, C++ / Python)</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Hudson River Trading</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr"/>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY (multiple) 2026-07-14</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>IMC Trading</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr"/>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Chicago, IL 2026-06-28</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Machine Learning Research Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>IMC Trading</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr"/>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Chicago, IL 2026-06-28</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (1) 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Kudu Dynamics</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr"/>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Chantilly, VA -</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (2) 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Kudu Dynamics</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr"/>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Chantilly, VA -</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (3) 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Kudu Dynamics</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr"/>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Chantilly, VA -</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Technical Intern, Software / Cyber / AI (Spring 2027, remote)</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>LA-Tech.org</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr"/>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA / Remote (US) 2026-07-09</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Pixel Serving</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>LiveRamp</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr"/>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY 2026-05-21</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Summer Intern (CS / Software / Engineering) 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>LufCo</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr"/>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Aberdeen, MD -</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern 🇺🇸 ⏳</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Naive</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr"/>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>San Francisco, CA / Remote (US) -</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Full Stack Engineering Intern 🇺🇸 ⏳</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Nash</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr"/>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>San Francisco, CA -</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Agent Platform / Full Stack (2026-2027)</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Netic</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr"/>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>San Francisco, CA 2026-07-16</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, BCI Applications ⏳</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Neuralink</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr"/>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Fremont, CA 2026-07-16</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (Summer 2027, June Start)</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Old Mission</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr"/>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Chicago, IL 2026-07-15</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (Austin)</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Optiver</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr"/>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Austin, TX 2026-06-28</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (Chicago)</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Optiver</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr"/>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Chicago, IL 2026-06-28</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (Summer 2027, grad 2028)</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Palantir</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr"/>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY (multiple US) 2026-07-09</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Infrastructure (Summer 2027, grad 2028)</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Palantir</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr"/>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY (multiple US) 2026-07-09</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Production Infrastructure (Summer 2027, grad 2028)</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Palantir</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr"/>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY (multiple US) 2026-07-09</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Defense Tech (Summer 2027, grad 2028)</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Palantir</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr"/>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Washington, DC (multiple US) 2026-07-09</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Forward Deployed Software Engineer Intern, Commercial (Summer 2027, grad Dec 2027 / Spring 2028)</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Palantir</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr"/>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY (multiple US) 2026-07-09</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>Year at Palantir, Forward Deployed Software Engineer Intern ⏳</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Palantir</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr"/>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY (multiple US) 2026-07-09</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern, Backend / Full Stack / ML (Winter 2027)</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Rippling</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr"/>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>San Francisco, CA / New York, NY / Seattle, WA 2026-06-27</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (Futureforce) 🔒</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr"/>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>San Francisco, CA -</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Electrical Engineering Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Second Order Effects</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr"/>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>El Segundo, CA / Redmond, WA 2026-07-19</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern (Fall 2026 / Winter 2027)</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Skydio</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr"/>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>San Mateo, CA 2026-05-06</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Stoke Space</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr"/>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>Kent, WA 2026-05-05</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>Quantitative Strategy Developer Intern (Summer 2027, June start)</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Susquehanna</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr"/>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Bala Cynwyd, PA -</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>Trading System Engineering Intern 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Susquehanna</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr"/>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>Bala Cynwyd, PA -</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern (North America, Summer 2027)</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>The Trade Desk</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr"/>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Denver, CO (multiple US) 2026-07-16</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Applied Scientist Intern, Monetization Technology (PhD, 2027 Start)</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr"/>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>San Jose, CA 2026-04-16</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>Quantitative Developer Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Tower Research Capital</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr"/>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY / Chicago, IL 2026-07-06</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Engineering Intern (12 roles: process, equipment, CIM / software)</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>TSMC Arizona</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr"/>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Phoenix, AZ 2026-06-04</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>AI Research Scientist Intern (MS / PhD)</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Two Sigma</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr"/>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>New York, NY 2026-07-08</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern (Summer 2027, Uber Career Prep)</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr"/>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>San Francisco, CA / Seattle, WA / Sunnyvale, CA 2026-07-20</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>Engineering Intern (Summer 2027) 🛂 🇺🇸</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Unison (GE Aerospace)</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr"/>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Jacksonville, FL 2026-07-16</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>Quantitative Developer Intern (2027)</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Voloridge Investment Management</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr"/>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>Jupiter, FL 2026-06-15</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>Quant Developer Intern</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Walleye Capital</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr"/>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>Boston, MA -</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Western Digital</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="inlineStr"/>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>San Jose, CA 2026-07-20</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>Postings (community list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>🔥 CLOSING SOON]</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>AWS Student Builder Group Leader — Deadline: Aug 16, 2026 (11:59 PM PST)</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr"/>
+      <c r="E98" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>AWS / NextGen</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>AWS Global University Program — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr"/>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>Base44</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>Campus Impact Leaders (Founding Class) — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr"/>
+      <c r="E100" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Canva</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>Campus Canvassadors (Founding Cohort, Aug–Dec 2026) — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr"/>
+      <c r="E101" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>🔥 CLOSING SOON]</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>CAVA</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>University of Minnesota Campus Brand Ambassador (Fall 2026) — Deadline: Aug 26, 2026</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr"/>
+      <c r="E102" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>⏳ OPENS SOON]</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="C103" s="6" t="inlineStr">
+        <is>
+          <t>Campus Expert — Deadline: Annual Window (Applications Open Each July; Next: July 2027)</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr"/>
+      <c r="E103" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
+          <t>Google Student Influencer Program (2026) — Deadline: Check site</t>
+        </is>
+      </c>
+      <c r="D104" s="5" t="inlineStr"/>
+      <c r="E104" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="inlineStr">
+        <is>
+          <t>Microsoft Learn Student Ambassadors — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr"/>
+      <c r="E105" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>Monster Energy</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>College Ambassador Team (CAT) — Deadline: Check site</t>
+        </is>
+      </c>
+      <c r="D106" s="5" t="inlineStr"/>
+      <c r="E106" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="inlineStr">
+        <is>
+          <t>OpenAI Student Collective (Campus Lead) — Deadline: Aug 31, 2026 (Japan, Korea, UK, Germany, France; US/Canada/India Cohort Closed)</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr"/>
+      <c r="E107" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>Pearson</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr">
+        <is>
+          <t>Pearson Campus Ambassador — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D108" s="5" t="inlineStr"/>
+      <c r="E108" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>Princess Polly</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="inlineStr">
+        <is>
+          <t>College Ambassador — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr"/>
+      <c r="E109" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F109" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>Red Bull</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>Student Marketeer — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D110" s="5" t="inlineStr"/>
+      <c r="E110" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>🔥 CLOSING SOON]</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="inlineStr">
+        <is>
+          <t>Uber Teen Ambassador (Seattle) — Deadline: Aug 15, 2026</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr"/>
+      <c r="E111" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>🔥 CLOSING SOON]</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>Uber Teen Ambassador (Phoenix) — Deadline: Aug 15, 2026</t>
+        </is>
+      </c>
+      <c r="D112" s="5" t="inlineStr"/>
+      <c r="E112" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>Walmart / Satya Blends</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="inlineStr">
+        <is>
+          <t>Walmart UGC Creator — Deadline: Check site</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr"/>
+      <c r="E113" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>Ambassador Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>Summer of Code</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="inlineStr">
+        <is>
+          <t>open-source, stipend, open to intl</t>
+        </is>
+      </c>
+      <c r="D114" s="5" t="inlineStr"/>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs always open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>Outreachy</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>Outreachy</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="inlineStr">
+        <is>
+          <t>open-source, stipend, open to intl</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr"/>
+      <c r="E115" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs always open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>Software Undergrad Engineering Internship</t>
+        </is>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>SWE intern (undergrad)</t>
+        </is>
+      </c>
+      <c r="D116" s="5" t="inlineStr">
+        <is>
+          <t>rolling</t>
+        </is>
+      </c>
+      <c r="E116" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs open now)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>Machine Learning &amp; AI Undergrad Internship</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="inlineStr">
+        <is>
+          <t>ML / AI intern (undergrad)</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>rolling</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs open now)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>Hardware Undergrad Engineering Internship</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="C118" s="6" t="inlineStr">
+        <is>
+          <t>hardware intern (undergrad)</t>
+        </is>
+      </c>
+      <c r="D118" s="5" t="inlineStr">
+        <is>
+          <t>rolling</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F118" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs open now)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>Student Fellows Program</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="inlineStr">
+        <is>
+          <t>data and AI fellowship</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>check site</t>
+        </is>
+      </c>
+      <c r="E119" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs open now)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>2027 US Summer Internship, Early Interest</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>Dexcom</t>
+        </is>
+      </c>
+      <c r="C120" s="6" t="inlineStr">
+        <is>
+          <t>early interest pipeline</t>
+        </is>
+      </c>
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>rolling</t>
+        </is>
+      </c>
+      <c r="E120" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F120" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs open now)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>Learn Student Ambassadors</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="C121" s="6" t="inlineStr">
+        <is>
+          <t>ambassador program</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>rolling</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F121" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs open now)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>MLH Fellowship</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>MLH</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="inlineStr">
+        <is>
+          <t>remote SWE fellowship, stipend</t>
+        </is>
+      </c>
+      <c r="D122" s="5" t="inlineStr">
+        <is>
+          <t>rolling</t>
+        </is>
+      </c>
+      <c r="E122" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs open now)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>Neo Scholars</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Neo</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="inlineStr">
+        <is>
+          <t>CS undergrad fellowship</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>approx June 14 to 30, 2026</t>
+        </is>
+      </c>
+      <c r="E123" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs open now)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>AI Builder, Emerging Talent</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="inlineStr">
+        <is>
+          <t>emerging talent program</t>
+        </is>
+      </c>
+      <c r="D124" s="5" t="inlineStr">
+        <is>
+          <t>check site</t>
+        </is>
+      </c>
+      <c r="E124" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs open now)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>2027 Summer Internships, Express Your Interest</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>Schonfeld</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="inlineStr">
+        <is>
+          <t>express interest pipeline, full roles open Aug 2026</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>rolling</t>
+        </is>
+      </c>
+      <c r="E125" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines (programs open now)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>Ayn Rand Institute</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="inlineStr">
+        <is>
+          <t>Fountainhead Essay Contest (Grades 11–12) — Deadline: Sep 13, 2026 (Anthem contest closed May 31, 2026)</t>
+        </is>
+      </c>
+      <c r="D126" s="5" t="inlineStr"/>
+      <c r="E126" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>Rising Freshmen &amp; Class of 2030 Opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>Coca-Cola Scholars Foundation</t>
+        </is>
+      </c>
+      <c r="C127" s="6" t="inlineStr">
+        <is>
+          <t>Coca-Cola Scholars Program (HS Senior; 3.0+ GPA)</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr"/>
+      <c r="E127" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F127" s="5" t="inlineStr">
+        <is>
+          <t>Rising Freshmen &amp; Class of 2030 Opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>Gates Foundation</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="inlineStr">
+        <is>
+          <t>The Gates Scholarship (Low-Income Minority HS Seniors)</t>
+        </is>
+      </c>
+      <c r="D128" s="5" t="inlineStr"/>
+      <c r="E128" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F128" s="5" t="inlineStr">
+        <is>
+          <t>Rising Freshmen &amp; Class of 2030 Opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>⏳ OPENS SOON]</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>Hagan Scholarship Foundation</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="inlineStr">
+        <is>
+          <t>Hagan Scholarship (HS Senior; 3.5+ GPA; Household Income ≤ $125K; 4-Yr Non-Profit College — No CC/Online)</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr"/>
+      <c r="E129" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F129" s="5" t="inlineStr">
+        <is>
+          <t>Rising Freshmen &amp; Class of 2030 Opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>Jane Street</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="inlineStr">
+        <is>
+          <t>WiSE - Women in Science &amp; Engineering (Class of 2030)</t>
+        </is>
+      </c>
+      <c r="D130" s="5" t="inlineStr"/>
+      <c r="E130" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F130" s="5" t="inlineStr">
+        <is>
+          <t>Rising Freshmen &amp; Class of 2030 Opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>National Merit Scholarship Corporation</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="inlineStr">
+        <is>
+          <t>National Merit Scholarship (PSAT/NMSQT Junior Year)</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr"/>
+      <c r="E131" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F131" s="5" t="inlineStr">
+        <is>
+          <t>Rising Freshmen &amp; Class of 2030 Opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>Optimist International</t>
+        </is>
+      </c>
+      <c r="C132" s="6" t="inlineStr">
+        <is>
+          <t>Optimist International Essay Contest (Under 19 on Oct 1; 700–800 word essay; 2026-27 topic announced)</t>
+        </is>
+      </c>
+      <c r="D132" s="5" t="inlineStr"/>
+      <c r="E132" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F132" s="5" t="inlineStr">
+        <is>
+          <t>Rising Freshmen &amp; Class of 2030 Opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Posse Foundation</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="inlineStr">
+        <is>
+          <t>Posse Scholarship (Nomination-Based; Partner Cities)</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="inlineStr"/>
+      <c r="E133" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F133" s="5" t="inlineStr">
+        <is>
+          <t>Rising Freshmen &amp; Class of 2030 Opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>QuestBridge</t>
+        </is>
+      </c>
+      <c r="C134" s="6" t="inlineStr">
+        <is>
+          <t>National College Match (HS Senior; Low-Income)</t>
+        </is>
+      </c>
+      <c r="D134" s="5" t="inlineStr"/>
+      <c r="E134" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F134" s="5" t="inlineStr">
+        <is>
+          <t>Rising Freshmen &amp; Class of 2030 Opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>Regeneron / Society for Science</t>
+        </is>
+      </c>
+      <c r="C135" s="6" t="inlineStr">
+        <is>
+          <t>Regeneron Science Talent Search (HS Senior STEM Research)</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr"/>
+      <c r="E135" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F135" s="5" t="inlineStr">
+        <is>
+          <t>Rising Freshmen &amp; Class of 2030 Opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="C136" s="6" t="inlineStr">
+        <is>
+          <t>Adobe NEXT// Campus Leader — Deadline: Check site</t>
+        </is>
+      </c>
+      <c r="D136" s="5" t="inlineStr"/>
+      <c r="E136" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F136" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>Career Pathways Initiative</t>
+        </is>
+      </c>
+      <c r="C137" s="6" t="inlineStr">
+        <is>
+          <t>Career Pathways Initiative Fellowship — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr"/>
+      <c r="E137" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F137" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>🔥 CLOSING SOON]</t>
+        </is>
+      </c>
+      <c r="B138" s="5" t="inlineStr">
+        <is>
+          <t>Coinbase</t>
+        </is>
+      </c>
+      <c r="C138" s="6" t="inlineStr">
+        <is>
+          <t>Next-Gen Networking — Deadline: Aug 19, 2026 (11:59 PM PT) (Event: Sep 2, 2026)</t>
+        </is>
+      </c>
+      <c r="D138" s="5" t="inlineStr"/>
+      <c r="E138" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F138" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+      <c r="C139" s="6" t="inlineStr">
+        <is>
+          <t>Databricks Student Fellows Program — Deadline: Check site</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr"/>
+      <c r="E139" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F139" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="C140" s="6" t="inlineStr">
+        <is>
+          <t>ElevenLabs Ambassador Program — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D140" s="5" t="inlineStr"/>
+      <c r="E140" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F140" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>GirlsWhoML</t>
+        </is>
+      </c>
+      <c r="C141" s="6" t="inlineStr">
+        <is>
+          <t>Thinking About Thinking 2026 Ambassador Programme — Deadline: Check site</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="inlineStr"/>
+      <c r="E141" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F141" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>Handshake</t>
+        </is>
+      </c>
+      <c r="C142" s="6" t="inlineStr">
+        <is>
+          <t>AI Fellowship Program — Deadline: Check site</t>
+        </is>
+      </c>
+      <c r="D142" s="5" t="inlineStr"/>
+      <c r="E142" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>🔥 CLOSING SOON]</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>HeadStart Fellowship</t>
+        </is>
+      </c>
+      <c r="C143" s="6" t="inlineStr">
+        <is>
+          <t>HeadStart Fellowship (Fall 2026) — Deadline: Aug 28, 2026 (11:59 PM ET)</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr"/>
+      <c r="E143" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>IOScholarships</t>
+        </is>
+      </c>
+      <c r="C144" s="6" t="inlineStr">
+        <is>
+          <t>AWS re/Start — Deadline: Rolling (Cohort: Sep 15–Dec 15, 2026)</t>
+        </is>
+      </c>
+      <c r="D144" s="5" t="inlineStr"/>
+      <c r="E144" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F144" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>Jane Street</t>
+        </is>
+      </c>
+      <c r="C145" s="6" t="inlineStr">
+        <is>
+          <t>FTTP — First-Year Trading &amp; Technology Program — Deadline: Rolling (Sign Up to Be Notified)</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr"/>
+      <c r="E145" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F145" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B146" s="5" t="inlineStr">
+        <is>
+          <t>Lime Connect</t>
+        </is>
+      </c>
+      <c r="C146" s="6" t="inlineStr">
+        <is>
+          <t>Lime Connect Network Membership — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D146" s="5" t="inlineStr"/>
+      <c r="E146" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F146" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>MLH (Major League Hacking)</t>
+        </is>
+      </c>
+      <c r="C147" s="6" t="inlineStr">
+        <is>
+          <t>MLH Fellowship — Deadline: Aug 31, 2026 (Fall Batch: Starts Sep 14, 2026)</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr"/>
+      <c r="E147" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F147" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="inlineStr">
+        <is>
+          <t>MLT (Management Leadership for Tomorrow)</t>
+        </is>
+      </c>
+      <c r="C148" s="6" t="inlineStr">
+        <is>
+          <t>MLT Career Prep (Class of 2029) — Deadline: Aug 1, 2026 – Jan 15, 2027 (Phased)</t>
+        </is>
+      </c>
+      <c r="D148" s="5" t="inlineStr"/>
+      <c r="E148" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F148" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>National Geographic Society × The Nature Conservancy</t>
+        </is>
+      </c>
+      <c r="C149" s="6" t="inlineStr">
+        <is>
+          <t>Community Conservation: Data Visualization &amp; Mapping Externship — Deadline: Aug 30, 2026</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr"/>
+      <c r="E149" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F149" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B150" s="5" t="inlineStr">
+        <is>
+          <t>NSN (National Sales Network)</t>
+        </is>
+      </c>
+      <c r="C150" s="6" t="inlineStr">
+        <is>
+          <t>2026 NSN Student Sales &amp; Marketing Conference — Deadline: Rolling (Event: Sep 12–14, 2026)</t>
+        </is>
+      </c>
+      <c r="D150" s="5" t="inlineStr"/>
+      <c r="E150" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F150" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>OpenTrade</t>
+        </is>
+      </c>
+      <c r="C151" s="6" t="inlineStr">
+        <is>
+          <t>OpenTrade Fellowship — Deadline: Rolling (Limited Spots)</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr"/>
+      <c r="E151" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F151" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B152" s="5" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="C152" s="6" t="inlineStr">
+        <is>
+          <t>PwC AI Externships — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D152" s="5" t="inlineStr"/>
+      <c r="E152" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F152" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>ServiceNow</t>
+        </is>
+      </c>
+      <c r="C153" s="6" t="inlineStr">
+        <is>
+          <t>Campus Leaders — Deadline: Rolling</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr"/>
+      <c r="E153" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B154" s="5" t="inlineStr">
+        <is>
+          <t>SHPE</t>
+        </is>
+      </c>
+      <c r="C154" s="6" t="inlineStr">
+        <is>
+          <t>2026 SHPE National Convention — Deadline: Check site (Event: Oct 28–31, 2026)</t>
+        </is>
+      </c>
+      <c r="D154" s="5" t="inlineStr"/>
+      <c r="E154" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F154" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>🔥 CLOSING SOON]</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>SoFi</t>
+        </is>
+      </c>
+      <c r="C155" s="6" t="inlineStr">
+        <is>
+          <t>SoFi Sophomore Externship 2026 — Deadline: Check site (Event: Aug 18–19, 2026)</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr"/>
+      <c r="E155" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>🔥 CLOSING SOON]</t>
+        </is>
+      </c>
+      <c r="B156" s="5" t="inlineStr">
+        <is>
+          <t>Stellic</t>
+        </is>
+      </c>
+      <c r="C156" s="6" t="inlineStr">
+        <is>
+          <t>The Pathfinders Challenge — Deadline: Aug 21, 2026 (Submissions Close)</t>
+        </is>
+      </c>
+      <c r="D156" s="5" t="inlineStr"/>
+      <c r="E156" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F156" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>The Home Depot</t>
+        </is>
+      </c>
+      <c r="C157" s="6" t="inlineStr">
+        <is>
+          <t>The Home Depot Externships (Multiple Tracks) — Deadline: Varies by Externship (Check Hub for Open Tracks)</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr"/>
+      <c r="E157" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F157" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>WomenHack</t>
+        </is>
+      </c>
+      <c r="C158" s="6" t="inlineStr">
+        <is>
+          <t>Women in Tech Career Fair — Deadline: Varies per event</t>
+        </is>
+      </c>
+      <c r="D158" s="5" t="inlineStr"/>
+      <c r="E158" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F158" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>🔥 CLOSING SOON]</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>Y Combinator</t>
+        </is>
+      </c>
+      <c r="C159" s="6" t="inlineStr">
+        <is>
+          <t>YC 2027 Summer Internship Expo — Deadline: Check site (Event: Aug 15, 2026)</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr"/>
+      <c r="E159" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Programs (Fellowships, Externships, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>✅ OPEN]</t>
+        </is>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C160" s="6" t="inlineStr">
+        <is>
+          <t>Student Researcher, BS/MS, Fall 2026 — Deadline: Nov 27, 2026 (Rolling; May Close Earlier)</t>
+        </is>
+      </c>
+      <c r="D160" s="5" t="inlineStr"/>
+      <c r="E160" s="7" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F160" s="5" t="inlineStr">
+        <is>
+          <t>Underclassmen Research Programs</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:F160"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E102" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E117" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E119" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E121" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E122" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E123" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E124" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E125" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E126" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E127" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E128" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E129" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E130" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E131" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E132" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E133" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E134" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E135" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E136" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E137" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E138" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E139" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E140" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E141" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E142" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E143" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E144" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E145" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E146" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E147" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E148" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E149" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E150" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E151" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E152" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E153" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E154" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E155" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E156" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E157" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E158" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E159" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E160" r:id="rId158"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>